<commit_message>
[DEV] database fixes, adjustment to return casket trips
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -16911,7 +16911,7 @@
         <v>1</v>
       </c>
       <c r="Q157" s="20" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="R157" s="23" t="s">
         <v>153</v>
@@ -18474,7 +18474,7 @@
         <v>1</v>
       </c>
       <c r="Q178" s="20" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="R178" s="23" t="s">
         <v>153</v>
@@ -19222,7 +19222,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="6" t="n">
         <v>82</v>
       </c>
@@ -19274,7 +19274,7 @@
       <c r="AF191" s="13"/>
       <c r="AG191" s="12"/>
     </row>
-    <row r="192" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="6" t="n">
         <v>83</v>
       </c>

</xml_diff>

<commit_message>
[DEV] cost approximations for outer shielding materials completed
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E0A3472-5308-4005-9264-C1E2F4072931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23F0D3E-B1DE-4E6C-8F51-F2F7C06F48B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="4185" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2944,18 +2944,13 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2965,13 +2960,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -5570,10 +5570,10 @@
       <c r="S3" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="123" t="s">
+      <c r="T3" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="U3" s="124" t="s">
+      <c r="U3" s="134" t="s">
         <v>42</v>
       </c>
       <c r="V3" s="2"/>
@@ -5669,8 +5669,8 @@
       <c r="S4" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="T4" s="123"/>
-      <c r="U4" s="123"/>
+      <c r="T4" s="132"/>
+      <c r="U4" s="132"/>
       <c r="V4" s="2"/>
       <c r="W4" s="19" t="s">
         <v>43</v>
@@ -5761,7 +5761,7 @@
       <c r="T5" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="U5" s="124" t="s">
+      <c r="U5" s="134" t="s">
         <v>58</v>
       </c>
       <c r="V5" s="2"/>
@@ -5853,7 +5853,7 @@
       <c r="T6" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="U6" s="124"/>
+      <c r="U6" s="134"/>
       <c r="V6" s="2"/>
       <c r="W6" s="19" t="s">
         <v>43</v>
@@ -6195,13 +6195,13 @@
       <c r="R11" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S11" s="123" t="s">
+      <c r="S11" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T11" s="123" t="s">
+      <c r="T11" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="125" t="s">
+      <c r="U11" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="2"/>
@@ -6294,9 +6294,9 @@
       <c r="R12" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S12" s="123"/>
-      <c r="T12" s="123"/>
-      <c r="U12" s="123"/>
+      <c r="S12" s="132"/>
+      <c r="T12" s="132"/>
+      <c r="U12" s="132"/>
       <c r="V12" s="2"/>
       <c r="W12" s="19" t="s">
         <v>77</v>
@@ -6387,9 +6387,9 @@
       <c r="R13" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S13" s="123"/>
-      <c r="T13" s="123"/>
-      <c r="U13" s="123"/>
+      <c r="S13" s="132"/>
+      <c r="T13" s="132"/>
+      <c r="U13" s="132"/>
       <c r="V13" s="2"/>
       <c r="W13" s="19" t="s">
         <v>77</v>
@@ -6518,13 +6518,13 @@
       <c r="R15" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S15" s="123" t="s">
+      <c r="S15" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T15" s="123" t="s">
+      <c r="T15" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U15" s="125" t="s">
+      <c r="U15" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V15" s="2"/>
@@ -6610,9 +6610,9 @@
       <c r="R16" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S16" s="123"/>
-      <c r="T16" s="123"/>
-      <c r="U16" s="123"/>
+      <c r="S16" s="132"/>
+      <c r="T16" s="132"/>
+      <c r="U16" s="132"/>
       <c r="V16" s="2"/>
       <c r="W16" s="19" t="s">
         <v>77</v>
@@ -6696,9 +6696,9 @@
       <c r="R17" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S17" s="123"/>
-      <c r="T17" s="123"/>
-      <c r="U17" s="123"/>
+      <c r="S17" s="132"/>
+      <c r="T17" s="132"/>
+      <c r="U17" s="132"/>
       <c r="V17" s="2"/>
       <c r="W17" s="19" t="s">
         <v>77</v>
@@ -7064,13 +7064,13 @@
       <c r="R22" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S22" s="123" t="s">
+      <c r="S22" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T22" s="123" t="s">
+      <c r="T22" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U22" s="125" t="s">
+      <c r="U22" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V22" s="2"/>
@@ -7156,9 +7156,9 @@
       <c r="R23" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S23" s="123"/>
-      <c r="T23" s="123"/>
-      <c r="U23" s="123"/>
+      <c r="S23" s="132"/>
+      <c r="T23" s="132"/>
+      <c r="U23" s="132"/>
       <c r="V23" s="2"/>
       <c r="W23" s="19" t="s">
         <v>77</v>
@@ -7242,9 +7242,9 @@
       <c r="R24" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S24" s="123"/>
-      <c r="T24" s="123"/>
-      <c r="U24" s="123"/>
+      <c r="S24" s="132"/>
+      <c r="T24" s="132"/>
+      <c r="U24" s="132"/>
       <c r="V24" s="2"/>
       <c r="W24" s="19" t="s">
         <v>77</v>
@@ -7373,13 +7373,13 @@
       <c r="R26" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S26" s="123" t="s">
+      <c r="S26" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T26" s="123" t="s">
+      <c r="T26" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U26" s="125" t="s">
+      <c r="U26" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V26" s="2"/>
@@ -7465,9 +7465,9 @@
       <c r="R27" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S27" s="123"/>
-      <c r="T27" s="123"/>
-      <c r="U27" s="123"/>
+      <c r="S27" s="132"/>
+      <c r="T27" s="132"/>
+      <c r="U27" s="132"/>
       <c r="V27" s="2"/>
       <c r="W27" s="19" t="s">
         <v>77</v>
@@ -7551,9 +7551,9 @@
       <c r="R28" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S28" s="123"/>
-      <c r="T28" s="123"/>
-      <c r="U28" s="123"/>
+      <c r="S28" s="132"/>
+      <c r="T28" s="132"/>
+      <c r="U28" s="132"/>
       <c r="V28" s="2"/>
       <c r="W28" s="19" t="s">
         <v>77</v>
@@ -7690,13 +7690,13 @@
       <c r="R30" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S30" s="123" t="s">
+      <c r="S30" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T30" s="123" t="s">
+      <c r="T30" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U30" s="125" t="s">
+      <c r="U30" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V30" s="2"/>
@@ -7786,9 +7786,9 @@
       <c r="R31" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S31" s="123"/>
-      <c r="T31" s="123"/>
-      <c r="U31" s="123"/>
+      <c r="S31" s="132"/>
+      <c r="T31" s="132"/>
+      <c r="U31" s="132"/>
       <c r="V31" s="2"/>
       <c r="W31" s="19" t="s">
         <v>77</v>
@@ -7876,9 +7876,9 @@
       <c r="R32" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S32" s="123"/>
-      <c r="T32" s="123"/>
-      <c r="U32" s="123"/>
+      <c r="S32" s="132"/>
+      <c r="T32" s="132"/>
+      <c r="U32" s="132"/>
       <c r="V32" s="2"/>
       <c r="W32" s="19" t="s">
         <v>77</v>
@@ -8197,13 +8197,13 @@
       <c r="R37" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S37" s="123" t="s">
+      <c r="S37" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T37" s="123" t="s">
+      <c r="T37" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U37" s="125" t="s">
+      <c r="U37" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V37" s="2"/>
@@ -8287,9 +8287,9 @@
       <c r="R38" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S38" s="123"/>
-      <c r="T38" s="123"/>
-      <c r="U38" s="123"/>
+      <c r="S38" s="132"/>
+      <c r="T38" s="132"/>
+      <c r="U38" s="132"/>
       <c r="V38" s="2"/>
       <c r="W38" s="19" t="s">
         <v>77</v>
@@ -8373,9 +8373,9 @@
       <c r="R39" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S39" s="123"/>
-      <c r="T39" s="123"/>
-      <c r="U39" s="123"/>
+      <c r="S39" s="132"/>
+      <c r="T39" s="132"/>
+      <c r="U39" s="132"/>
       <c r="V39" s="2"/>
       <c r="W39" s="19" t="s">
         <v>77</v>
@@ -8504,13 +8504,13 @@
       <c r="R41" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S41" s="123" t="s">
+      <c r="S41" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T41" s="123" t="s">
+      <c r="T41" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U41" s="125" t="s">
+      <c r="U41" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V41" s="2"/>
@@ -8596,9 +8596,9 @@
       <c r="R42" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S42" s="123"/>
-      <c r="T42" s="123"/>
-      <c r="U42" s="123"/>
+      <c r="S42" s="132"/>
+      <c r="T42" s="132"/>
+      <c r="U42" s="132"/>
       <c r="V42" s="2"/>
       <c r="W42" s="19" t="s">
         <v>77</v>
@@ -8682,9 +8682,9 @@
       <c r="R43" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S43" s="123"/>
-      <c r="T43" s="123"/>
-      <c r="U43" s="123"/>
+      <c r="S43" s="132"/>
+      <c r="T43" s="132"/>
+      <c r="U43" s="132"/>
       <c r="V43" s="2"/>
       <c r="W43" s="19" t="s">
         <v>77</v>
@@ -8865,13 +8865,13 @@
       <c r="R46" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S46" s="123" t="s">
+      <c r="S46" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T46" s="123" t="s">
+      <c r="T46" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U46" s="125" t="s">
+      <c r="U46" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V46" s="2"/>
@@ -8957,9 +8957,9 @@
       <c r="R47" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S47" s="123"/>
-      <c r="T47" s="123"/>
-      <c r="U47" s="123"/>
+      <c r="S47" s="132"/>
+      <c r="T47" s="132"/>
+      <c r="U47" s="132"/>
       <c r="V47" s="2"/>
       <c r="W47" s="19" t="s">
         <v>77</v>
@@ -9043,9 +9043,9 @@
       <c r="R48" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S48" s="123"/>
-      <c r="T48" s="123"/>
-      <c r="U48" s="123"/>
+      <c r="S48" s="132"/>
+      <c r="T48" s="132"/>
+      <c r="U48" s="132"/>
       <c r="V48" s="2"/>
       <c r="W48" s="19" t="s">
         <v>77</v>
@@ -9316,16 +9316,16 @@
       <c r="R52" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S52" s="123" t="s">
+      <c r="S52" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T52" s="123" t="s">
+      <c r="T52" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="125" t="s">
+      <c r="U52" s="133" t="s">
         <v>76</v>
       </c>
-      <c r="V52" s="126" t="s">
+      <c r="V52" s="131" t="s">
         <v>162</v>
       </c>
       <c r="W52" s="19" t="s">
@@ -9410,10 +9410,10 @@
       <c r="R53" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="S53" s="123"/>
-      <c r="T53" s="123"/>
-      <c r="U53" s="123"/>
-      <c r="V53" s="126"/>
+      <c r="S53" s="132"/>
+      <c r="T53" s="132"/>
+      <c r="U53" s="132"/>
+      <c r="V53" s="131"/>
       <c r="W53" s="19" t="s">
         <v>77</v>
       </c>
@@ -9496,10 +9496,10 @@
       <c r="R54" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S54" s="123"/>
-      <c r="T54" s="123"/>
-      <c r="U54" s="123"/>
-      <c r="V54" s="126"/>
+      <c r="S54" s="132"/>
+      <c r="T54" s="132"/>
+      <c r="U54" s="132"/>
+      <c r="V54" s="131"/>
       <c r="W54" s="19" t="s">
         <v>77</v>
       </c>
@@ -9672,13 +9672,13 @@
       <c r="R57" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S57" s="123" t="s">
+      <c r="S57" s="132" t="s">
         <v>105</v>
       </c>
-      <c r="T57" s="123" t="s">
+      <c r="T57" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="125" t="s">
+      <c r="U57" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="2"/>
@@ -9764,9 +9764,9 @@
       <c r="R58" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S58" s="123"/>
-      <c r="T58" s="123"/>
-      <c r="U58" s="123"/>
+      <c r="S58" s="132"/>
+      <c r="T58" s="132"/>
+      <c r="U58" s="132"/>
       <c r="V58" s="2"/>
       <c r="W58" s="19" t="s">
         <v>77</v>
@@ -9850,9 +9850,9 @@
       <c r="R59" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S59" s="123"/>
-      <c r="T59" s="123"/>
-      <c r="U59" s="123"/>
+      <c r="S59" s="132"/>
+      <c r="T59" s="132"/>
+      <c r="U59" s="132"/>
       <c r="V59" s="2"/>
       <c r="W59" s="19" t="s">
         <v>77</v>
@@ -9981,13 +9981,13 @@
       <c r="R61" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S61" s="123" t="s">
+      <c r="S61" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T61" s="123" t="s">
+      <c r="T61" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U61" s="125" t="s">
+      <c r="U61" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V61" s="2"/>
@@ -10073,9 +10073,9 @@
       <c r="R62" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S62" s="123"/>
-      <c r="T62" s="123"/>
-      <c r="U62" s="123"/>
+      <c r="S62" s="132"/>
+      <c r="T62" s="132"/>
+      <c r="U62" s="132"/>
       <c r="V62" s="2"/>
       <c r="W62" s="19" t="s">
         <v>77</v>
@@ -10159,9 +10159,9 @@
       <c r="R63" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S63" s="123"/>
-      <c r="T63" s="123"/>
-      <c r="U63" s="123"/>
+      <c r="S63" s="132"/>
+      <c r="T63" s="132"/>
+      <c r="U63" s="132"/>
       <c r="V63" s="2"/>
       <c r="W63" s="19" t="s">
         <v>77</v>
@@ -10485,7 +10485,7 @@
       <c r="S68" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T68" s="127" t="s">
+      <c r="T68" s="128" t="s">
         <v>197</v>
       </c>
       <c r="U68" s="38"/>
@@ -10576,7 +10576,7 @@
       <c r="S69" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T69" s="127"/>
+      <c r="T69" s="128"/>
       <c r="U69" s="38"/>
       <c r="V69" s="2"/>
       <c r="W69" s="19" t="s">
@@ -10672,7 +10672,7 @@
       <c r="S70" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T70" s="127"/>
+      <c r="T70" s="128"/>
       <c r="U70" s="38"/>
       <c r="V70" s="2"/>
       <c r="W70" s="19" t="s">
@@ -10775,7 +10775,7 @@
       <c r="S71" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T71" s="127"/>
+      <c r="T71" s="128"/>
       <c r="U71" s="38"/>
       <c r="V71" s="30" t="s">
         <v>203</v>
@@ -10873,7 +10873,7 @@
       <c r="S72" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T72" s="127"/>
+      <c r="T72" s="128"/>
       <c r="U72" s="38"/>
       <c r="V72" s="30"/>
       <c r="W72" s="19" t="s">
@@ -10969,7 +10969,7 @@
       <c r="S73" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="T73" s="127"/>
+      <c r="T73" s="128"/>
       <c r="U73" s="38"/>
       <c r="V73" s="30"/>
       <c r="W73" s="19" t="s">
@@ -11166,10 +11166,10 @@
       <c r="S76" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="T76" s="127" t="s">
+      <c r="T76" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="U76" s="128" t="s">
+      <c r="U76" s="129" t="s">
         <v>211</v>
       </c>
       <c r="V76" s="30" t="s">
@@ -11265,8 +11265,8 @@
       <c r="S77" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="T77" s="127"/>
-      <c r="U77" s="127"/>
+      <c r="T77" s="128"/>
+      <c r="U77" s="128"/>
       <c r="V77" s="2"/>
       <c r="W77" s="19" t="s">
         <v>213</v>
@@ -11369,8 +11369,8 @@
       <c r="S78" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="T78" s="127"/>
-      <c r="U78" s="127"/>
+      <c r="T78" s="128"/>
+      <c r="U78" s="128"/>
       <c r="V78" s="2"/>
       <c r="W78" s="19" t="s">
         <v>157</v>
@@ -11465,8 +11465,8 @@
       <c r="S79" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="T79" s="127"/>
-      <c r="U79" s="127"/>
+      <c r="T79" s="128"/>
+      <c r="U79" s="128"/>
       <c r="V79" s="2"/>
       <c r="W79" s="19" t="s">
         <v>157</v>
@@ -11569,8 +11569,8 @@
       <c r="S80" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="T80" s="127"/>
-      <c r="U80" s="127"/>
+      <c r="T80" s="128"/>
+      <c r="U80" s="128"/>
       <c r="V80" s="2"/>
       <c r="W80" s="19" t="s">
         <v>226</v>
@@ -12084,7 +12084,7 @@
       <c r="T86" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="U86" s="129" t="s">
+      <c r="U86" s="130" t="s">
         <v>211</v>
       </c>
       <c r="V86" s="2"/>
@@ -12192,7 +12192,7 @@
       <c r="T87" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="U87" s="129"/>
+      <c r="U87" s="130"/>
       <c r="V87" s="2"/>
       <c r="W87" s="19" t="s">
         <v>226</v>
@@ -12298,7 +12298,7 @@
       <c r="T88" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="U88" s="129"/>
+      <c r="U88" s="130"/>
       <c r="V88" s="2"/>
       <c r="W88" s="19" t="s">
         <v>228</v>
@@ -12395,7 +12395,7 @@
       <c r="T89" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="U89" s="129"/>
+      <c r="U89" s="130"/>
       <c r="V89" s="2"/>
       <c r="W89" s="19" t="s">
         <v>228</v>
@@ -12486,7 +12486,7 @@
       <c r="T90" s="30" t="s">
         <v>231</v>
       </c>
-      <c r="U90" s="129"/>
+      <c r="U90" s="130"/>
       <c r="V90" s="2"/>
       <c r="W90" s="19" t="s">
         <v>157</v>
@@ -12577,7 +12577,7 @@
       <c r="T91" s="30" t="s">
         <v>231</v>
       </c>
-      <c r="U91" s="129"/>
+      <c r="U91" s="130"/>
       <c r="V91" s="2"/>
       <c r="W91" s="19" t="s">
         <v>157</v>
@@ -12666,7 +12666,7 @@
         <v>242</v>
       </c>
       <c r="T92" s="30"/>
-      <c r="U92" s="129"/>
+      <c r="U92" s="130"/>
       <c r="V92" s="2"/>
       <c r="W92" s="19" t="s">
         <v>157</v>
@@ -12755,7 +12755,7 @@
         <v>242</v>
       </c>
       <c r="T93" s="30"/>
-      <c r="U93" s="129"/>
+      <c r="U93" s="130"/>
       <c r="V93" s="2"/>
       <c r="W93" s="19" t="s">
         <v>157</v>
@@ -12844,7 +12844,7 @@
         <v>244</v>
       </c>
       <c r="T94" s="30"/>
-      <c r="U94" s="129"/>
+      <c r="U94" s="130"/>
       <c r="V94" s="2" t="s">
         <v>245</v>
       </c>
@@ -12938,7 +12938,7 @@
         <v>244</v>
       </c>
       <c r="T95" s="30"/>
-      <c r="U95" s="129"/>
+      <c r="U95" s="130"/>
       <c r="V95" s="2" t="s">
         <v>245</v>
       </c>
@@ -13032,7 +13032,7 @@
         <v>247</v>
       </c>
       <c r="T96" s="30"/>
-      <c r="U96" s="129"/>
+      <c r="U96" s="130"/>
       <c r="V96" s="2" t="s">
         <v>245</v>
       </c>
@@ -13533,7 +13533,7 @@
       <c r="J102" s="23"/>
       <c r="K102" s="24">
         <f t="shared" ref="K102:K109" si="19">(AA102+AB102)/2</f>
-        <v>215</v>
+        <v>607.5</v>
       </c>
       <c r="L102" s="2" t="s">
         <v>186</v>
@@ -13583,10 +13583,10 @@
         <v>44</v>
       </c>
       <c r="AA102" s="58">
-        <v>150</v>
+        <v>375</v>
       </c>
       <c r="AB102" s="58">
-        <v>280</v>
+        <v>840</v>
       </c>
       <c r="AC102" s="19" t="s">
         <v>44</v>
@@ -13632,8 +13632,8 @@
       <c r="I103" s="17"/>
       <c r="J103" s="23"/>
       <c r="K103" s="24">
-        <f t="shared" si="19"/>
-        <v>430</v>
+        <f>(AA103+AB103)/2</f>
+        <v>1160</v>
       </c>
       <c r="L103" s="2" t="s">
         <v>186</v>
@@ -13683,10 +13683,10 @@
         <v>44</v>
       </c>
       <c r="AA103" s="58">
-        <v>260</v>
+        <v>520</v>
       </c>
       <c r="AB103" s="58">
-        <v>600</v>
+        <v>1800</v>
       </c>
       <c r="AC103" s="19" t="s">
         <v>44</v>
@@ -13733,7 +13733,7 @@
       <c r="J104" s="23"/>
       <c r="K104" s="24">
         <f t="shared" si="19"/>
-        <v>440</v>
+        <v>1185</v>
       </c>
       <c r="L104" s="2" t="s">
         <v>186</v>
@@ -13783,10 +13783,10 @@
         <v>44</v>
       </c>
       <c r="AA104" s="58">
-        <v>270</v>
+        <v>540</v>
       </c>
       <c r="AB104" s="58">
-        <v>610</v>
+        <v>1830</v>
       </c>
       <c r="AC104" s="19" t="s">
         <v>44</v>
@@ -13833,7 +13833,7 @@
       <c r="J105" s="23"/>
       <c r="K105" s="24">
         <f t="shared" si="19"/>
-        <v>737.5</v>
+        <v>2005</v>
       </c>
       <c r="L105" s="2" t="s">
         <v>186</v>
@@ -13883,10 +13883,10 @@
         <v>44</v>
       </c>
       <c r="AA105" s="58">
-        <v>415</v>
+        <v>830</v>
       </c>
       <c r="AB105" s="58">
-        <v>1060</v>
+        <v>3180</v>
       </c>
       <c r="AC105" s="19" t="s">
         <v>44</v>
@@ -13933,7 +13933,7 @@
       <c r="J106" s="23"/>
       <c r="K106" s="24">
         <f t="shared" si="19"/>
-        <v>215</v>
+        <v>607.5</v>
       </c>
       <c r="L106" s="2" t="s">
         <v>186</v>
@@ -13983,10 +13983,10 @@
         <v>44</v>
       </c>
       <c r="AA106" s="58">
-        <v>150</v>
+        <v>375</v>
       </c>
       <c r="AB106" s="58">
-        <v>280</v>
+        <v>840</v>
       </c>
       <c r="AC106" s="19" t="s">
         <v>44</v>
@@ -14033,7 +14033,7 @@
       <c r="J107" s="23"/>
       <c r="K107" s="24">
         <f t="shared" si="19"/>
-        <v>430</v>
+        <v>1160</v>
       </c>
       <c r="L107" s="2" t="s">
         <v>186</v>
@@ -14083,10 +14083,10 @@
         <v>44</v>
       </c>
       <c r="AA107" s="58">
-        <v>260</v>
+        <v>520</v>
       </c>
       <c r="AB107" s="58">
-        <v>600</v>
+        <v>1800</v>
       </c>
       <c r="AC107" s="19" t="s">
         <v>44</v>
@@ -14133,7 +14133,7 @@
       <c r="J108" s="23"/>
       <c r="K108" s="24">
         <f t="shared" si="19"/>
-        <v>440</v>
+        <v>1185</v>
       </c>
       <c r="L108" s="2" t="s">
         <v>186</v>
@@ -14183,10 +14183,10 @@
         <v>44</v>
       </c>
       <c r="AA108" s="58">
-        <v>270</v>
+        <v>540</v>
       </c>
       <c r="AB108" s="58">
-        <v>610</v>
+        <v>1830</v>
       </c>
       <c r="AC108" s="19" t="s">
         <v>44</v>
@@ -14233,7 +14233,7 @@
       <c r="J109" s="23"/>
       <c r="K109" s="24">
         <f t="shared" si="19"/>
-        <v>737.5</v>
+        <v>2005</v>
       </c>
       <c r="L109" s="2" t="s">
         <v>186</v>
@@ -14283,10 +14283,10 @@
         <v>44</v>
       </c>
       <c r="AA109" s="58">
-        <v>415</v>
+        <v>830</v>
       </c>
       <c r="AB109" s="58">
-        <v>1060</v>
+        <v>3180</v>
       </c>
       <c r="AC109" s="19" t="s">
         <v>44</v>
@@ -14737,9 +14737,9 @@
       <c r="S114" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="T114" s="127"/>
-      <c r="U114" s="130"/>
-      <c r="V114" s="130"/>
+      <c r="T114" s="128"/>
+      <c r="U114" s="126"/>
+      <c r="V114" s="126"/>
       <c r="W114" s="19" t="s">
         <v>157</v>
       </c>
@@ -14824,9 +14824,9 @@
       <c r="S115" s="30" t="s">
         <v>271</v>
       </c>
-      <c r="T115" s="127"/>
-      <c r="U115" s="130"/>
-      <c r="V115" s="130"/>
+      <c r="T115" s="128"/>
+      <c r="U115" s="126"/>
+      <c r="V115" s="126"/>
       <c r="W115" s="19" t="s">
         <v>157</v>
       </c>
@@ -15937,7 +15937,7 @@
       <c r="S128" s="30"/>
       <c r="T128" s="2"/>
       <c r="U128" s="2"/>
-      <c r="V128" s="134"/>
+      <c r="V128" s="127"/>
       <c r="W128" s="19"/>
       <c r="X128" s="28"/>
       <c r="Y128" s="28"/>
@@ -16011,7 +16011,7 @@
         <v>309</v>
       </c>
       <c r="U129" s="2"/>
-      <c r="V129" s="134"/>
+      <c r="V129" s="127"/>
       <c r="W129" s="19" t="s">
         <v>157</v>
       </c>
@@ -17194,10 +17194,10 @@
       <c r="R143" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S143" s="132" t="s">
+      <c r="S143" s="124" t="s">
         <v>336</v>
       </c>
-      <c r="T143" s="133" t="s">
+      <c r="T143" s="125" t="s">
         <v>337</v>
       </c>
       <c r="U143" s="53" t="s">
@@ -17288,8 +17288,8 @@
       <c r="R144" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="S144" s="132"/>
-      <c r="T144" s="132"/>
+      <c r="S144" s="124"/>
+      <c r="T144" s="124"/>
       <c r="U144" s="53" t="s">
         <v>341</v>
       </c>
@@ -17379,8 +17379,8 @@
       <c r="R145" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S145" s="132"/>
-      <c r="T145" s="132"/>
+      <c r="S145" s="124"/>
+      <c r="T145" s="124"/>
       <c r="U145" s="2"/>
       <c r="V145" s="2"/>
       <c r="W145" s="19" t="s">
@@ -17450,8 +17450,8 @@
       <c r="P146" s="2"/>
       <c r="Q146" s="27"/>
       <c r="R146" s="2"/>
-      <c r="S146" s="132"/>
-      <c r="T146" s="132"/>
+      <c r="S146" s="124"/>
+      <c r="T146" s="124"/>
       <c r="U146" s="2"/>
       <c r="V146" s="2"/>
       <c r="W146" s="19"/>
@@ -17495,8 +17495,8 @@
       <c r="P147" s="2"/>
       <c r="Q147" s="27"/>
       <c r="R147" s="2"/>
-      <c r="S147" s="132"/>
-      <c r="T147" s="132"/>
+      <c r="S147" s="124"/>
+      <c r="T147" s="124"/>
       <c r="U147" s="2"/>
       <c r="V147" s="2"/>
       <c r="W147" s="19"/>
@@ -17556,8 +17556,8 @@
       <c r="R148" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S148" s="132"/>
-      <c r="T148" s="132"/>
+      <c r="S148" s="124"/>
+      <c r="T148" s="124"/>
       <c r="U148" s="53" t="s">
         <v>349</v>
       </c>
@@ -17694,8 +17694,8 @@
       <c r="P150" s="2"/>
       <c r="Q150" s="27"/>
       <c r="R150" s="2"/>
-      <c r="S150" s="132"/>
-      <c r="T150" s="133"/>
+      <c r="S150" s="124"/>
+      <c r="T150" s="125"/>
       <c r="U150" s="2"/>
       <c r="V150" s="2"/>
       <c r="W150" s="19"/>
@@ -17758,8 +17758,8 @@
       <c r="R151" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S151" s="132"/>
-      <c r="T151" s="132"/>
+      <c r="S151" s="124"/>
+      <c r="T151" s="124"/>
       <c r="U151" s="2"/>
       <c r="V151" s="2"/>
       <c r="W151" s="19" t="s">
@@ -17846,8 +17846,8 @@
       <c r="R152" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S152" s="132"/>
-      <c r="T152" s="132"/>
+      <c r="S152" s="124"/>
+      <c r="T152" s="124"/>
       <c r="U152" s="2"/>
       <c r="V152" s="2"/>
       <c r="W152" s="19" t="s">
@@ -17934,8 +17934,8 @@
       <c r="R153" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S153" s="132"/>
-      <c r="T153" s="132"/>
+      <c r="S153" s="124"/>
+      <c r="T153" s="124"/>
       <c r="U153" s="2"/>
       <c r="V153" s="2"/>
       <c r="W153" s="19" t="s">
@@ -18022,8 +18022,8 @@
       <c r="R154" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S154" s="132"/>
-      <c r="T154" s="132"/>
+      <c r="S154" s="124"/>
+      <c r="T154" s="124"/>
       <c r="U154" s="2"/>
       <c r="V154" s="2"/>
       <c r="W154" s="19" t="s">
@@ -18110,8 +18110,8 @@
       <c r="R155" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S155" s="132"/>
-      <c r="T155" s="132"/>
+      <c r="S155" s="124"/>
+      <c r="T155" s="124"/>
       <c r="U155" s="2"/>
       <c r="V155" s="2"/>
       <c r="W155" s="19" t="s">
@@ -18496,7 +18496,7 @@
       <c r="R160" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S160" s="131"/>
+      <c r="S160" s="123"/>
       <c r="T160" s="1"/>
       <c r="U160" s="2"/>
       <c r="V160" s="2"/>
@@ -18587,7 +18587,7 @@
       <c r="R161" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S161" s="131"/>
+      <c r="S161" s="123"/>
       <c r="T161" s="1"/>
       <c r="U161" s="2"/>
       <c r="V161" s="2"/>
@@ -18685,7 +18685,7 @@
       <c r="R162" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S162" s="131"/>
+      <c r="S162" s="123"/>
       <c r="T162" s="1"/>
       <c r="U162" s="2"/>
       <c r="V162" s="2"/>
@@ -18779,7 +18779,7 @@
       <c r="R163" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S163" s="131"/>
+      <c r="S163" s="123"/>
       <c r="T163" s="47"/>
       <c r="U163" s="2"/>
       <c r="V163" s="2"/>
@@ -19825,12 +19825,12 @@
       <c r="R179" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S179" s="132"/>
-      <c r="T179" s="132" t="s">
+      <c r="S179" s="124"/>
+      <c r="T179" s="124" t="s">
         <v>400</v>
       </c>
       <c r="U179" s="2"/>
-      <c r="V179" s="133"/>
+      <c r="V179" s="125"/>
       <c r="W179" s="19" t="s">
         <v>43</v>
       </c>
@@ -19916,10 +19916,10 @@
       <c r="R180" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S180" s="132"/>
-      <c r="T180" s="132"/>
+      <c r="S180" s="124"/>
+      <c r="T180" s="124"/>
       <c r="U180" s="2"/>
-      <c r="V180" s="133"/>
+      <c r="V180" s="125"/>
       <c r="W180" s="19" t="s">
         <v>43</v>
       </c>
@@ -20005,10 +20005,10 @@
       <c r="R181" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S181" s="132"/>
-      <c r="T181" s="132"/>
+      <c r="S181" s="124"/>
+      <c r="T181" s="124"/>
       <c r="U181" s="2"/>
-      <c r="V181" s="133"/>
+      <c r="V181" s="125"/>
       <c r="W181" s="19" t="s">
         <v>43</v>
       </c>
@@ -20093,10 +20093,10 @@
       <c r="R182" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S182" s="132"/>
-      <c r="T182" s="132"/>
+      <c r="S182" s="124"/>
+      <c r="T182" s="124"/>
       <c r="U182" s="2"/>
-      <c r="V182" s="133"/>
+      <c r="V182" s="125"/>
       <c r="W182" s="19" t="s">
         <v>43</v>
       </c>
@@ -20164,10 +20164,10 @@
       <c r="P183" s="2"/>
       <c r="Q183" s="27"/>
       <c r="R183" s="2"/>
-      <c r="S183" s="132"/>
-      <c r="T183" s="132"/>
+      <c r="S183" s="124"/>
+      <c r="T183" s="124"/>
       <c r="U183" s="2"/>
-      <c r="V183" s="133"/>
+      <c r="V183" s="125"/>
       <c r="W183" s="19"/>
       <c r="X183" s="28"/>
       <c r="Y183" s="28"/>
@@ -20227,12 +20227,12 @@
       <c r="R184" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S184" s="132"/>
-      <c r="T184" s="132"/>
+      <c r="S184" s="124"/>
+      <c r="T184" s="124"/>
       <c r="U184" s="52" t="s">
         <v>319</v>
       </c>
-      <c r="V184" s="133"/>
+      <c r="V184" s="125"/>
       <c r="W184" s="19" t="s">
         <v>43</v>
       </c>
@@ -20325,10 +20325,10 @@
       <c r="R185" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S185" s="132"/>
-      <c r="T185" s="132"/>
+      <c r="S185" s="124"/>
+      <c r="T185" s="124"/>
       <c r="U185" s="52"/>
-      <c r="V185" s="133"/>
+      <c r="V185" s="125"/>
       <c r="W185" s="19" t="s">
         <v>43</v>
       </c>
@@ -21505,6 +21505,49 @@
   </sheetData>
   <autoFilter ref="A1:AB189" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="53">
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="S11:S13"/>
+    <mergeCell ref="T11:T13"/>
+    <mergeCell ref="U11:U13"/>
+    <mergeCell ref="S15:S17"/>
+    <mergeCell ref="T15:T17"/>
+    <mergeCell ref="U15:U17"/>
+    <mergeCell ref="S22:S24"/>
+    <mergeCell ref="T22:T24"/>
+    <mergeCell ref="U22:U24"/>
+    <mergeCell ref="S26:S28"/>
+    <mergeCell ref="T26:T28"/>
+    <mergeCell ref="U26:U28"/>
+    <mergeCell ref="S30:S32"/>
+    <mergeCell ref="T30:T32"/>
+    <mergeCell ref="U30:U32"/>
+    <mergeCell ref="S37:S39"/>
+    <mergeCell ref="T37:T39"/>
+    <mergeCell ref="U37:U39"/>
+    <mergeCell ref="S41:S43"/>
+    <mergeCell ref="T41:T43"/>
+    <mergeCell ref="U41:U43"/>
+    <mergeCell ref="S46:S48"/>
+    <mergeCell ref="T46:T48"/>
+    <mergeCell ref="U46:U48"/>
+    <mergeCell ref="S52:S54"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="V52:V54"/>
+    <mergeCell ref="S57:S59"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="U57:U59"/>
+    <mergeCell ref="S61:S63"/>
+    <mergeCell ref="T61:T63"/>
+    <mergeCell ref="U61:U63"/>
+    <mergeCell ref="T68:T73"/>
+    <mergeCell ref="T76:T80"/>
+    <mergeCell ref="U76:U80"/>
+    <mergeCell ref="U86:U96"/>
+    <mergeCell ref="T114:T115"/>
+    <mergeCell ref="U114:U115"/>
     <mergeCell ref="S160:S163"/>
     <mergeCell ref="S179:S185"/>
     <mergeCell ref="T179:T185"/>
@@ -21515,49 +21558,6 @@
     <mergeCell ref="T143:T148"/>
     <mergeCell ref="S150:S155"/>
     <mergeCell ref="T150:T155"/>
-    <mergeCell ref="T68:T73"/>
-    <mergeCell ref="T76:T80"/>
-    <mergeCell ref="U76:U80"/>
-    <mergeCell ref="U86:U96"/>
-    <mergeCell ref="T114:T115"/>
-    <mergeCell ref="U114:U115"/>
-    <mergeCell ref="V52:V54"/>
-    <mergeCell ref="S57:S59"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="U57:U59"/>
-    <mergeCell ref="S61:S63"/>
-    <mergeCell ref="T61:T63"/>
-    <mergeCell ref="U61:U63"/>
-    <mergeCell ref="S46:S48"/>
-    <mergeCell ref="T46:T48"/>
-    <mergeCell ref="U46:U48"/>
-    <mergeCell ref="S52:S54"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="S37:S39"/>
-    <mergeCell ref="T37:T39"/>
-    <mergeCell ref="U37:U39"/>
-    <mergeCell ref="S41:S43"/>
-    <mergeCell ref="T41:T43"/>
-    <mergeCell ref="U41:U43"/>
-    <mergeCell ref="S26:S28"/>
-    <mergeCell ref="T26:T28"/>
-    <mergeCell ref="U26:U28"/>
-    <mergeCell ref="S30:S32"/>
-    <mergeCell ref="T30:T32"/>
-    <mergeCell ref="U30:U32"/>
-    <mergeCell ref="S15:S17"/>
-    <mergeCell ref="T15:T17"/>
-    <mergeCell ref="U15:U17"/>
-    <mergeCell ref="S22:S24"/>
-    <mergeCell ref="T22:T24"/>
-    <mergeCell ref="U22:U24"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="S11:S13"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="U11:U13"/>
   </mergeCells>
   <conditionalFormatting sqref="A97:B101">
     <cfRule type="expression" dxfId="302" priority="197">
@@ -26124,10 +26124,10 @@
       <c r="S3" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="123" t="s">
+      <c r="T3" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="U3" s="124" t="s">
+      <c r="U3" s="134" t="s">
         <v>42</v>
       </c>
       <c r="V3" s="2"/>
@@ -26227,8 +26227,8 @@
       <c r="S4" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="T4" s="123"/>
-      <c r="U4" s="123"/>
+      <c r="T4" s="132"/>
+      <c r="U4" s="132"/>
       <c r="V4" s="2"/>
       <c r="W4" s="19" t="s">
         <v>43</v>
@@ -26320,10 +26320,10 @@
       <c r="S5" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="T5" s="123" t="s">
+      <c r="T5" s="132" t="s">
         <v>63</v>
       </c>
-      <c r="U5" s="124" t="s">
+      <c r="U5" s="134" t="s">
         <v>58</v>
       </c>
       <c r="V5" s="2"/>
@@ -26416,8 +26416,8 @@
       <c r="S6" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="T6" s="123"/>
-      <c r="U6" s="123"/>
+      <c r="T6" s="132"/>
+      <c r="U6" s="132"/>
       <c r="V6" s="2"/>
       <c r="W6" s="19" t="s">
         <v>43</v>
@@ -26767,13 +26767,13 @@
       <c r="R11" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S11" s="123" t="s">
+      <c r="S11" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T11" s="123" t="s">
+      <c r="T11" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="125" t="s">
+      <c r="U11" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="2"/>
@@ -26870,9 +26870,9 @@
       <c r="R12" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S12" s="123"/>
-      <c r="T12" s="123"/>
-      <c r="U12" s="123"/>
+      <c r="S12" s="132"/>
+      <c r="T12" s="132"/>
+      <c r="U12" s="132"/>
       <c r="V12" s="2"/>
       <c r="W12" s="19" t="s">
         <v>43</v>
@@ -26967,9 +26967,9 @@
       <c r="R13" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="S13" s="123"/>
-      <c r="T13" s="123"/>
-      <c r="U13" s="123"/>
+      <c r="S13" s="132"/>
+      <c r="T13" s="132"/>
+      <c r="U13" s="132"/>
       <c r="V13" s="2"/>
       <c r="W13" s="19" t="s">
         <v>43</v>
@@ -27320,13 +27320,13 @@
       <c r="R18" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S18" s="123" t="s">
+      <c r="S18" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T18" s="123" t="s">
+      <c r="T18" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U18" s="125" t="s">
+      <c r="U18" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V18" s="2"/>
@@ -27418,9 +27418,9 @@
       <c r="R19" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S19" s="123"/>
-      <c r="T19" s="123"/>
-      <c r="U19" s="123"/>
+      <c r="S19" s="132"/>
+      <c r="T19" s="132"/>
+      <c r="U19" s="132"/>
       <c r="V19" s="2"/>
       <c r="W19" s="19" t="s">
         <v>43</v>
@@ -27510,9 +27510,9 @@
       <c r="R20" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S20" s="123"/>
-      <c r="T20" s="123"/>
-      <c r="U20" s="123"/>
+      <c r="S20" s="132"/>
+      <c r="T20" s="132"/>
+      <c r="U20" s="132"/>
       <c r="V20" s="2"/>
       <c r="W20" s="19" t="s">
         <v>43</v>
@@ -27731,13 +27731,13 @@
       <c r="R23" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S23" s="123" t="s">
+      <c r="S23" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T23" s="123" t="s">
+      <c r="T23" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U23" s="125" t="s">
+      <c r="U23" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V23" s="2"/>
@@ -27829,9 +27829,9 @@
       <c r="R24" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S24" s="123"/>
-      <c r="T24" s="123"/>
-      <c r="U24" s="123"/>
+      <c r="S24" s="132"/>
+      <c r="T24" s="132"/>
+      <c r="U24" s="132"/>
       <c r="V24" s="2"/>
       <c r="W24" s="19" t="s">
         <v>43</v>
@@ -27921,9 +27921,9 @@
       <c r="R25" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S25" s="123"/>
-      <c r="T25" s="123"/>
-      <c r="U25" s="123"/>
+      <c r="S25" s="132"/>
+      <c r="T25" s="132"/>
+      <c r="U25" s="132"/>
       <c r="V25" s="2"/>
       <c r="W25" s="19" t="s">
         <v>43</v>
@@ -28142,13 +28142,13 @@
       <c r="R28" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S28" s="123" t="s">
+      <c r="S28" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T28" s="123" t="s">
+      <c r="T28" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U28" s="125" t="s">
+      <c r="U28" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V28" s="2"/>
@@ -28240,9 +28240,9 @@
       <c r="R29" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S29" s="123"/>
-      <c r="T29" s="123"/>
-      <c r="U29" s="123"/>
+      <c r="S29" s="132"/>
+      <c r="T29" s="132"/>
+      <c r="U29" s="132"/>
       <c r="V29" s="2"/>
       <c r="W29" s="19" t="s">
         <v>43</v>
@@ -28332,9 +28332,9 @@
       <c r="R30" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S30" s="123"/>
-      <c r="T30" s="123"/>
-      <c r="U30" s="123"/>
+      <c r="S30" s="132"/>
+      <c r="T30" s="132"/>
+      <c r="U30" s="132"/>
       <c r="V30" s="2"/>
       <c r="W30" s="19" t="s">
         <v>43</v>
@@ -28553,13 +28553,13 @@
       <c r="R33" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S33" s="123" t="s">
+      <c r="S33" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T33" s="123" t="s">
+      <c r="T33" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U33" s="125" t="s">
+      <c r="U33" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V33" s="2"/>
@@ -28651,9 +28651,9 @@
       <c r="R34" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S34" s="123"/>
-      <c r="T34" s="123"/>
-      <c r="U34" s="123"/>
+      <c r="S34" s="132"/>
+      <c r="T34" s="132"/>
+      <c r="U34" s="132"/>
       <c r="V34" s="2"/>
       <c r="W34" s="19" t="s">
         <v>43</v>
@@ -28743,9 +28743,9 @@
       <c r="R35" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S35" s="123"/>
-      <c r="T35" s="123"/>
-      <c r="U35" s="123"/>
+      <c r="S35" s="132"/>
+      <c r="T35" s="132"/>
+      <c r="U35" s="132"/>
       <c r="V35" s="2"/>
       <c r="W35" s="19" t="s">
         <v>43</v>
@@ -28964,13 +28964,13 @@
       <c r="R38" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S38" s="123" t="s">
+      <c r="S38" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T38" s="123" t="s">
+      <c r="T38" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U38" s="125" t="s">
+      <c r="U38" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V38" s="2"/>
@@ -29062,9 +29062,9 @@
       <c r="R39" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S39" s="123"/>
-      <c r="T39" s="123"/>
-      <c r="U39" s="123"/>
+      <c r="S39" s="132"/>
+      <c r="T39" s="132"/>
+      <c r="U39" s="132"/>
       <c r="V39" s="2"/>
       <c r="W39" s="19" t="s">
         <v>43</v>
@@ -29154,9 +29154,9 @@
       <c r="R40" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S40" s="123"/>
-      <c r="T40" s="123"/>
-      <c r="U40" s="123"/>
+      <c r="S40" s="132"/>
+      <c r="T40" s="132"/>
+      <c r="U40" s="132"/>
       <c r="V40" s="2"/>
       <c r="W40" s="19" t="s">
         <v>43</v>
@@ -29514,13 +29514,13 @@
       <c r="R45" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S45" s="123" t="s">
+      <c r="S45" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T45" s="123" t="s">
+      <c r="T45" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U45" s="125" t="s">
+      <c r="U45" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V45" s="2"/>
@@ -29612,9 +29612,9 @@
       <c r="R46" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S46" s="123"/>
-      <c r="T46" s="123"/>
-      <c r="U46" s="123"/>
+      <c r="S46" s="132"/>
+      <c r="T46" s="132"/>
+      <c r="U46" s="132"/>
       <c r="V46" s="2"/>
       <c r="W46" s="19" t="s">
         <v>43</v>
@@ -29704,9 +29704,9 @@
       <c r="R47" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S47" s="123"/>
-      <c r="T47" s="123"/>
-      <c r="U47" s="123"/>
+      <c r="S47" s="132"/>
+      <c r="T47" s="132"/>
+      <c r="U47" s="132"/>
       <c r="V47" s="2"/>
       <c r="W47" s="19" t="s">
         <v>43</v>
@@ -30072,13 +30072,13 @@
       <c r="R52" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S52" s="123" t="s">
+      <c r="S52" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T52" s="123" t="s">
+      <c r="T52" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="125" t="s">
+      <c r="U52" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V52" s="2"/>
@@ -30170,9 +30170,9 @@
       <c r="R53" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S53" s="123"/>
-      <c r="T53" s="123"/>
-      <c r="U53" s="123"/>
+      <c r="S53" s="132"/>
+      <c r="T53" s="132"/>
+      <c r="U53" s="132"/>
       <c r="V53" s="2"/>
       <c r="W53" s="19" t="s">
         <v>43</v>
@@ -30262,9 +30262,9 @@
       <c r="R54" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S54" s="123"/>
-      <c r="T54" s="123"/>
-      <c r="U54" s="123"/>
+      <c r="S54" s="132"/>
+      <c r="T54" s="132"/>
+      <c r="U54" s="132"/>
       <c r="V54" s="2"/>
       <c r="W54" s="19" t="s">
         <v>43</v>
@@ -30495,13 +30495,13 @@
       <c r="R57" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S57" s="123" t="s">
+      <c r="S57" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T57" s="123" t="s">
+      <c r="T57" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="125" t="s">
+      <c r="U57" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="2"/>
@@ -30593,9 +30593,9 @@
       <c r="R58" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S58" s="123"/>
-      <c r="T58" s="123"/>
-      <c r="U58" s="123"/>
+      <c r="S58" s="132"/>
+      <c r="T58" s="132"/>
+      <c r="U58" s="132"/>
       <c r="V58" s="2"/>
       <c r="W58" s="19" t="s">
         <v>43</v>
@@ -30685,9 +30685,9 @@
       <c r="R59" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S59" s="123"/>
-      <c r="T59" s="123"/>
-      <c r="U59" s="123"/>
+      <c r="S59" s="132"/>
+      <c r="T59" s="132"/>
+      <c r="U59" s="132"/>
       <c r="V59" s="2"/>
       <c r="W59" s="19" t="s">
         <v>43</v>
@@ -30906,13 +30906,13 @@
       <c r="R62" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S62" s="123" t="s">
+      <c r="S62" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T62" s="123" t="s">
+      <c r="T62" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U62" s="125" t="s">
+      <c r="U62" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V62" s="2"/>
@@ -31004,9 +31004,9 @@
       <c r="R63" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S63" s="123"/>
-      <c r="T63" s="123"/>
-      <c r="U63" s="123"/>
+      <c r="S63" s="132"/>
+      <c r="T63" s="132"/>
+      <c r="U63" s="132"/>
       <c r="V63" s="2"/>
       <c r="W63" s="19" t="s">
         <v>43</v>
@@ -31096,9 +31096,9 @@
       <c r="R64" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S64" s="123"/>
-      <c r="T64" s="123"/>
-      <c r="U64" s="123"/>
+      <c r="S64" s="132"/>
+      <c r="T64" s="132"/>
+      <c r="U64" s="132"/>
       <c r="V64" s="2"/>
       <c r="W64" s="19" t="s">
         <v>43</v>
@@ -31317,13 +31317,13 @@
       <c r="R67" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S67" s="123" t="s">
+      <c r="S67" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T67" s="123" t="s">
+      <c r="T67" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U67" s="125" t="s">
+      <c r="U67" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V67" s="2"/>
@@ -31415,9 +31415,9 @@
       <c r="R68" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S68" s="123"/>
-      <c r="T68" s="123"/>
-      <c r="U68" s="123"/>
+      <c r="S68" s="132"/>
+      <c r="T68" s="132"/>
+      <c r="U68" s="132"/>
       <c r="V68" s="2"/>
       <c r="W68" s="19" t="s">
         <v>43</v>
@@ -31507,9 +31507,9 @@
       <c r="R69" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S69" s="123"/>
-      <c r="T69" s="123"/>
-      <c r="U69" s="123"/>
+      <c r="S69" s="132"/>
+      <c r="T69" s="132"/>
+      <c r="U69" s="132"/>
       <c r="V69" s="2"/>
       <c r="W69" s="19" t="s">
         <v>43</v>
@@ -31867,13 +31867,13 @@
       <c r="R74" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S74" s="123" t="s">
+      <c r="S74" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T74" s="123" t="s">
+      <c r="T74" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U74" s="125" t="s">
+      <c r="U74" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V74" s="2"/>
@@ -31965,9 +31965,9 @@
       <c r="R75" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S75" s="123"/>
-      <c r="T75" s="123"/>
-      <c r="U75" s="123"/>
+      <c r="S75" s="132"/>
+      <c r="T75" s="132"/>
+      <c r="U75" s="132"/>
       <c r="V75" s="2"/>
       <c r="W75" s="19" t="s">
         <v>43</v>
@@ -32057,9 +32057,9 @@
       <c r="R76" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S76" s="123"/>
-      <c r="T76" s="123"/>
-      <c r="U76" s="123"/>
+      <c r="S76" s="132"/>
+      <c r="T76" s="132"/>
+      <c r="U76" s="132"/>
       <c r="V76" s="2"/>
       <c r="W76" s="19" t="s">
         <v>43</v>
@@ -32278,13 +32278,13 @@
       <c r="R79" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S79" s="123" t="s">
+      <c r="S79" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T79" s="123" t="s">
+      <c r="T79" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U79" s="125" t="s">
+      <c r="U79" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V79" s="2"/>
@@ -32376,9 +32376,9 @@
       <c r="R80" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S80" s="123"/>
-      <c r="T80" s="123"/>
-      <c r="U80" s="123"/>
+      <c r="S80" s="132"/>
+      <c r="T80" s="132"/>
+      <c r="U80" s="132"/>
       <c r="V80" s="2"/>
       <c r="W80" s="19" t="s">
         <v>43</v>
@@ -32468,9 +32468,9 @@
       <c r="R81" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S81" s="123"/>
-      <c r="T81" s="123"/>
-      <c r="U81" s="123"/>
+      <c r="S81" s="132"/>
+      <c r="T81" s="132"/>
+      <c r="U81" s="132"/>
       <c r="V81" s="2"/>
       <c r="W81" s="19" t="s">
         <v>43</v>
@@ -32841,13 +32841,13 @@
       <c r="R86" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S86" s="123" t="s">
+      <c r="S86" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T86" s="123" t="s">
+      <c r="T86" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U86" s="125" t="s">
+      <c r="U86" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V86" s="2"/>
@@ -32939,9 +32939,9 @@
       <c r="R87" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S87" s="123"/>
-      <c r="T87" s="123"/>
-      <c r="U87" s="123"/>
+      <c r="S87" s="132"/>
+      <c r="T87" s="132"/>
+      <c r="U87" s="132"/>
       <c r="V87" s="2"/>
       <c r="W87" s="19" t="s">
         <v>43</v>
@@ -33031,9 +33031,9 @@
       <c r="R88" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S88" s="123"/>
-      <c r="T88" s="123"/>
-      <c r="U88" s="123"/>
+      <c r="S88" s="132"/>
+      <c r="T88" s="132"/>
+      <c r="U88" s="132"/>
       <c r="V88" s="2"/>
       <c r="W88" s="19" t="s">
         <v>43</v>
@@ -33400,13 +33400,13 @@
       <c r="R93" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S93" s="123" t="s">
+      <c r="S93" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T93" s="123" t="s">
+      <c r="T93" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U93" s="125" t="s">
+      <c r="U93" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V93" s="2"/>
@@ -33498,9 +33498,9 @@
       <c r="R94" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S94" s="123"/>
-      <c r="T94" s="123"/>
-      <c r="U94" s="123"/>
+      <c r="S94" s="132"/>
+      <c r="T94" s="132"/>
+      <c r="U94" s="132"/>
       <c r="V94" s="2"/>
       <c r="W94" s="19" t="s">
         <v>43</v>
@@ -33590,9 +33590,9 @@
       <c r="R95" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S95" s="123"/>
-      <c r="T95" s="123"/>
-      <c r="U95" s="123"/>
+      <c r="S95" s="132"/>
+      <c r="T95" s="132"/>
+      <c r="U95" s="132"/>
       <c r="V95" s="2"/>
       <c r="W95" s="19" t="s">
         <v>43</v>
@@ -33811,13 +33811,13 @@
       <c r="R98" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S98" s="123" t="s">
+      <c r="S98" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T98" s="123" t="s">
+      <c r="T98" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U98" s="125" t="s">
+      <c r="U98" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V98" s="2"/>
@@ -33909,9 +33909,9 @@
       <c r="R99" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S99" s="123"/>
-      <c r="T99" s="123"/>
-      <c r="U99" s="123"/>
+      <c r="S99" s="132"/>
+      <c r="T99" s="132"/>
+      <c r="U99" s="132"/>
       <c r="V99" s="2"/>
       <c r="W99" s="19" t="s">
         <v>43</v>
@@ -34001,9 +34001,9 @@
       <c r="R100" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S100" s="123"/>
-      <c r="T100" s="123"/>
-      <c r="U100" s="123"/>
+      <c r="S100" s="132"/>
+      <c r="T100" s="132"/>
+      <c r="U100" s="132"/>
       <c r="V100" s="2"/>
       <c r="W100" s="19" t="s">
         <v>43</v>
@@ -34382,13 +34382,13 @@
       <c r="R105" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S105" s="123" t="s">
+      <c r="S105" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T105" s="123" t="s">
+      <c r="T105" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U105" s="125" t="s">
+      <c r="U105" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V105" s="2"/>
@@ -34487,9 +34487,9 @@
       <c r="R106" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S106" s="123"/>
-      <c r="T106" s="123"/>
-      <c r="U106" s="123"/>
+      <c r="S106" s="132"/>
+      <c r="T106" s="132"/>
+      <c r="U106" s="132"/>
       <c r="V106" s="2"/>
       <c r="W106" s="19" t="s">
         <v>43</v>
@@ -34579,9 +34579,9 @@
       <c r="R107" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S107" s="123"/>
-      <c r="T107" s="123"/>
-      <c r="U107" s="123"/>
+      <c r="S107" s="132"/>
+      <c r="T107" s="132"/>
+      <c r="U107" s="132"/>
       <c r="V107" s="2"/>
       <c r="W107" s="19" t="s">
         <v>43</v>
@@ -34953,13 +34953,13 @@
       <c r="R112" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S112" s="123" t="s">
+      <c r="S112" s="132" t="s">
         <v>74</v>
       </c>
-      <c r="T112" s="123" t="s">
+      <c r="T112" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U112" s="125" t="s">
+      <c r="U112" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V112" s="2"/>
@@ -35051,9 +35051,9 @@
       <c r="R113" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S113" s="123"/>
-      <c r="T113" s="123"/>
-      <c r="U113" s="123"/>
+      <c r="S113" s="132"/>
+      <c r="T113" s="132"/>
+      <c r="U113" s="132"/>
       <c r="V113" s="2"/>
       <c r="W113" s="19" t="s">
         <v>43</v>
@@ -35143,9 +35143,9 @@
       <c r="R114" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S114" s="123"/>
-      <c r="T114" s="123"/>
-      <c r="U114" s="123"/>
+      <c r="S114" s="132"/>
+      <c r="T114" s="132"/>
+      <c r="U114" s="132"/>
       <c r="V114" s="2"/>
       <c r="W114" s="19" t="s">
         <v>43</v>
@@ -35377,13 +35377,13 @@
       <c r="R117" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S117" s="123" t="s">
+      <c r="S117" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T117" s="123" t="s">
+      <c r="T117" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U117" s="125" t="s">
+      <c r="U117" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V117" s="2"/>
@@ -35482,9 +35482,9 @@
       <c r="R118" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S118" s="123"/>
-      <c r="T118" s="123"/>
-      <c r="U118" s="123"/>
+      <c r="S118" s="132"/>
+      <c r="T118" s="132"/>
+      <c r="U118" s="132"/>
       <c r="V118" s="2"/>
       <c r="W118" s="19" t="s">
         <v>43</v>
@@ -35581,9 +35581,9 @@
       <c r="R119" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S119" s="123"/>
-      <c r="T119" s="123"/>
-      <c r="U119" s="123"/>
+      <c r="S119" s="132"/>
+      <c r="T119" s="132"/>
+      <c r="U119" s="132"/>
       <c r="V119" s="2"/>
       <c r="W119" s="19" t="s">
         <v>43</v>
@@ -35816,13 +35816,13 @@
       <c r="R122" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S122" s="123" t="s">
+      <c r="S122" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T122" s="123" t="s">
+      <c r="T122" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U122" s="125" t="s">
+      <c r="U122" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V122" s="2"/>
@@ -35914,9 +35914,9 @@
       <c r="R123" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S123" s="123"/>
-      <c r="T123" s="123"/>
-      <c r="U123" s="123"/>
+      <c r="S123" s="132"/>
+      <c r="T123" s="132"/>
+      <c r="U123" s="132"/>
       <c r="V123" s="2"/>
       <c r="W123" s="19" t="s">
         <v>43</v>
@@ -36006,9 +36006,9 @@
       <c r="R124" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S124" s="123"/>
-      <c r="T124" s="123"/>
-      <c r="U124" s="123"/>
+      <c r="S124" s="132"/>
+      <c r="T124" s="132"/>
+      <c r="U124" s="132"/>
       <c r="V124" s="2"/>
       <c r="W124" s="19" t="s">
         <v>43</v>
@@ -36227,13 +36227,13 @@
       <c r="R127" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S127" s="123" t="s">
+      <c r="S127" s="132" t="s">
         <v>603</v>
       </c>
-      <c r="T127" s="123" t="s">
+      <c r="T127" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="U127" s="125" t="s">
+      <c r="U127" s="133" t="s">
         <v>76</v>
       </c>
       <c r="V127" s="2"/>
@@ -36325,9 +36325,9 @@
       <c r="R128" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S128" s="123"/>
-      <c r="T128" s="123"/>
-      <c r="U128" s="123"/>
+      <c r="S128" s="132"/>
+      <c r="T128" s="132"/>
+      <c r="U128" s="132"/>
       <c r="V128" s="2"/>
       <c r="W128" s="19" t="s">
         <v>43</v>
@@ -36417,9 +36417,9 @@
       <c r="R129" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="S129" s="123"/>
-      <c r="T129" s="123"/>
-      <c r="U129" s="123"/>
+      <c r="S129" s="132"/>
+      <c r="T129" s="132"/>
+      <c r="U129" s="132"/>
       <c r="V129" s="2"/>
       <c r="W129" s="19" t="s">
         <v>43</v>
@@ -43650,10 +43650,10 @@
       <c r="R225" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S225" s="127" t="s">
+      <c r="S225" s="128" t="s">
         <v>710</v>
       </c>
-      <c r="T225" s="127" t="s">
+      <c r="T225" s="128" t="s">
         <v>711</v>
       </c>
       <c r="U225" s="2"/>
@@ -43736,8 +43736,8 @@
       <c r="R226" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S226" s="127"/>
-      <c r="T226" s="127"/>
+      <c r="S226" s="128"/>
+      <c r="T226" s="128"/>
       <c r="U226" s="2"/>
       <c r="V226" s="2"/>
       <c r="W226" s="19" t="s">
@@ -43825,8 +43825,8 @@
       <c r="R227" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S227" s="127"/>
-      <c r="T227" s="127"/>
+      <c r="S227" s="128"/>
+      <c r="T227" s="128"/>
       <c r="U227" s="2"/>
       <c r="V227" s="2"/>
       <c r="W227" s="19" t="s">
@@ -43914,8 +43914,8 @@
       <c r="R228" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S228" s="127"/>
-      <c r="T228" s="127"/>
+      <c r="S228" s="128"/>
+      <c r="T228" s="128"/>
       <c r="U228" s="2"/>
       <c r="V228" s="2"/>
       <c r="W228" s="19" t="s">
@@ -43996,8 +43996,8 @@
       <c r="R229" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S229" s="127"/>
-      <c r="T229" s="127"/>
+      <c r="S229" s="128"/>
+      <c r="T229" s="128"/>
       <c r="U229" s="2"/>
       <c r="V229" s="2"/>
       <c r="W229" s="19" t="s">
@@ -44078,8 +44078,8 @@
       <c r="R230" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S230" s="127"/>
-      <c r="T230" s="127"/>
+      <c r="S230" s="128"/>
+      <c r="T230" s="128"/>
       <c r="U230" s="2"/>
       <c r="V230" s="2"/>
       <c r="W230" s="19" t="s">
@@ -44838,7 +44838,7 @@
       <c r="R242" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="S242" s="123" t="s">
+      <c r="S242" s="132" t="s">
         <v>333</v>
       </c>
       <c r="T242" s="26"/>
@@ -44896,7 +44896,7 @@
       <c r="R243" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="S243" s="123"/>
+      <c r="S243" s="132"/>
       <c r="T243" s="26"/>
       <c r="U243" s="26"/>
       <c r="V243" s="26"/>
@@ -44960,7 +44960,7 @@
       <c r="R244" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S244" s="123"/>
+      <c r="S244" s="132"/>
       <c r="T244" s="2"/>
       <c r="U244" s="2"/>
       <c r="V244" s="2"/>
@@ -45017,7 +45017,7 @@
       <c r="R245" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S245" s="123"/>
+      <c r="S245" s="132"/>
       <c r="T245" s="2"/>
       <c r="U245" s="2"/>
       <c r="V245" s="2"/>
@@ -46422,11 +46422,61 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="S225:S230"/>
-    <mergeCell ref="T225:T230"/>
-    <mergeCell ref="S242:S245"/>
-    <mergeCell ref="S122:S124"/>
-    <mergeCell ref="T122:T124"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="S11:S13"/>
+    <mergeCell ref="T11:T13"/>
+    <mergeCell ref="U11:U13"/>
+    <mergeCell ref="S18:S20"/>
+    <mergeCell ref="T18:T20"/>
+    <mergeCell ref="U18:U20"/>
+    <mergeCell ref="S23:S25"/>
+    <mergeCell ref="T23:T25"/>
+    <mergeCell ref="U23:U25"/>
+    <mergeCell ref="S28:S30"/>
+    <mergeCell ref="T28:T30"/>
+    <mergeCell ref="U28:U30"/>
+    <mergeCell ref="S33:S35"/>
+    <mergeCell ref="T33:T35"/>
+    <mergeCell ref="U33:U35"/>
+    <mergeCell ref="S38:S40"/>
+    <mergeCell ref="T38:T40"/>
+    <mergeCell ref="U38:U40"/>
+    <mergeCell ref="S45:S47"/>
+    <mergeCell ref="T45:T47"/>
+    <mergeCell ref="U45:U47"/>
+    <mergeCell ref="S52:S54"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="S57:S59"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="U57:U59"/>
+    <mergeCell ref="S62:S64"/>
+    <mergeCell ref="T62:T64"/>
+    <mergeCell ref="U62:U64"/>
+    <mergeCell ref="S67:S69"/>
+    <mergeCell ref="T67:T69"/>
+    <mergeCell ref="U67:U69"/>
+    <mergeCell ref="S74:S76"/>
+    <mergeCell ref="T74:T76"/>
+    <mergeCell ref="U74:U76"/>
+    <mergeCell ref="S79:S81"/>
+    <mergeCell ref="T79:T81"/>
+    <mergeCell ref="U79:U81"/>
+    <mergeCell ref="S86:S88"/>
+    <mergeCell ref="T86:T88"/>
+    <mergeCell ref="U86:U88"/>
+    <mergeCell ref="S93:S95"/>
+    <mergeCell ref="T93:T95"/>
+    <mergeCell ref="U93:U95"/>
+    <mergeCell ref="S98:S100"/>
+    <mergeCell ref="T98:T100"/>
+    <mergeCell ref="U98:U100"/>
+    <mergeCell ref="S105:S107"/>
+    <mergeCell ref="T105:T107"/>
+    <mergeCell ref="U105:U107"/>
     <mergeCell ref="U122:U124"/>
     <mergeCell ref="S127:S129"/>
     <mergeCell ref="T127:T129"/>
@@ -46437,61 +46487,11 @@
     <mergeCell ref="S117:S119"/>
     <mergeCell ref="T117:T119"/>
     <mergeCell ref="U117:U119"/>
-    <mergeCell ref="S98:S100"/>
-    <mergeCell ref="T98:T100"/>
-    <mergeCell ref="U98:U100"/>
-    <mergeCell ref="S105:S107"/>
-    <mergeCell ref="T105:T107"/>
-    <mergeCell ref="U105:U107"/>
-    <mergeCell ref="S86:S88"/>
-    <mergeCell ref="T86:T88"/>
-    <mergeCell ref="U86:U88"/>
-    <mergeCell ref="S93:S95"/>
-    <mergeCell ref="T93:T95"/>
-    <mergeCell ref="U93:U95"/>
-    <mergeCell ref="S74:S76"/>
-    <mergeCell ref="T74:T76"/>
-    <mergeCell ref="U74:U76"/>
-    <mergeCell ref="S79:S81"/>
-    <mergeCell ref="T79:T81"/>
-    <mergeCell ref="U79:U81"/>
-    <mergeCell ref="S62:S64"/>
-    <mergeCell ref="T62:T64"/>
-    <mergeCell ref="U62:U64"/>
-    <mergeCell ref="S67:S69"/>
-    <mergeCell ref="T67:T69"/>
-    <mergeCell ref="U67:U69"/>
-    <mergeCell ref="S52:S54"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="S57:S59"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="U57:U59"/>
-    <mergeCell ref="S38:S40"/>
-    <mergeCell ref="T38:T40"/>
-    <mergeCell ref="U38:U40"/>
-    <mergeCell ref="S45:S47"/>
-    <mergeCell ref="T45:T47"/>
-    <mergeCell ref="U45:U47"/>
-    <mergeCell ref="S28:S30"/>
-    <mergeCell ref="T28:T30"/>
-    <mergeCell ref="U28:U30"/>
-    <mergeCell ref="S33:S35"/>
-    <mergeCell ref="T33:T35"/>
-    <mergeCell ref="U33:U35"/>
-    <mergeCell ref="S18:S20"/>
-    <mergeCell ref="T18:T20"/>
-    <mergeCell ref="U18:U20"/>
-    <mergeCell ref="S23:S25"/>
-    <mergeCell ref="T23:T25"/>
-    <mergeCell ref="U23:U25"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="T5:T6"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="S11:S13"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="U11:U13"/>
+    <mergeCell ref="S225:S230"/>
+    <mergeCell ref="T225:T230"/>
+    <mergeCell ref="S242:S245"/>
+    <mergeCell ref="S122:S124"/>
+    <mergeCell ref="T122:T124"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>